<commit_message>
fixed powerpoint size too large, error in pushing to git
</commit_message>
<xml_diff>
--- a/week-01/Ex3C_SurveyResults.xlsx
+++ b/week-01/Ex3C_SurveyResults.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\angelosorio\Documents\DataAnalytics\week-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1AD3B1A-CC00-449F-8780-9CEC373A5118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C44BA915-CFB5-454A-9A46-C4A6743BB9F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
+    <sheet name="GamblingStats" sheetId="3" r:id="rId1"/>
+    <sheet name="Survey" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="66">
   <si>
     <t>Id</t>
   </si>
@@ -231,16 +231,13 @@
     <t>Time To Complete</t>
   </si>
   <si>
-    <t>=COUNTIF(J2:J9, "Somewhat satisfied")</t>
-  </si>
-  <si>
     <t>Row Labels</t>
   </si>
   <si>
     <t>Grand Total</t>
   </si>
   <si>
-    <t>=countif([Are you a gambler?], "Yes" )</t>
+    <t>Count of Name</t>
   </si>
 </sst>
 </file>
@@ -248,7 +245,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="m/d/yyyy\ h:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="m/d/yyyy\ h:mm:ss"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -298,31 +295,93 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="45" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="35">
+  <dxfs count="33">
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="double">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="double">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -340,40 +399,10 @@
       <numFmt numFmtId="28" formatCode="mm:ss"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <numFmt numFmtId="164" formatCode="m/d/yyyy\ h:mm:ss"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="28" formatCode="mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="m/d/yyyy\ h:mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="m/d/yyyy\ h:mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="28" formatCode="mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="m/d/yyyy\ h:mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="m/d/yyyy\ h:mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="164" formatCode="m/d/yyyy\ h:mm:ss"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -420,6 +449,18 @@
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="28" formatCode="mm:ss"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m/d/yyyy\ h:mm:ss"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m/d/yyyy\ h:mm:ss"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -447,17 +488,777 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Ex3C_SurveyResults.xlsx]Sheet2!PivotTable1</c:name>
+    <c:name>[Ex3C_SurveyResults.xlsx]GamblingStats!PivotTable2</c:name>
     <c:fmtId val="0"/>
   </c:pivotSource>
   <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
     <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>GamblingStats!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-EF97-46D0-87EA-2C3E26A00135}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-EF97-46D0-87EA-2C3E26A00135}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-EF97-46D0-87EA-2C3E26A00135}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>GamblingStats!$A$2:$A$5</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Maybe</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>No</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Yes</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>GamblingStats!$B$2:$B$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-687E-484A-B047-B70E526D791C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+        <c14:dropZonesVisible val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[Ex3C_SurveyResults.xlsx]GamblingStats!PivotTable2</c:name>
+    <c:fmtId val="8"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="4"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="5"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="6"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="7"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="8"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+    </c:pivotFmts>
     <c:plotArea>
       <c:layout/>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
         <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>GamblingStats!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-AD8F-4534-9623-B21D4300A4FF}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-AD8F-4534-9623-B21D4300A4FF}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-AD8F-4534-9623-B21D4300A4FF}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>GamblingStats!$A$2:$A$5</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Maybe</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>No</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Yes</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>GamblingStats!$B$2:$B$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000006-AD8F-4534-9623-B21D4300A4FF}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
@@ -466,19 +1267,19 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:gapWidth val="219"/>
-        <c:overlap val="-27"/>
-        <c:axId val="30175087"/>
-        <c:axId val="30176527"/>
+        <c:gapWidth val="100"/>
+        <c:axId val="1601737775"/>
+        <c:axId val="1601737295"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="30175087"/>
+        <c:axId val="1601737775"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:majorTickMark val="none"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -514,7 +1315,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30176527"/>
+        <c:crossAx val="1601737295"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -522,7 +1323,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="30176527"/>
+        <c:axId val="1601737295"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -542,7 +1343,8 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:majorTickMark val="none"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -572,7 +1374,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30175087"/>
+        <c:crossAx val="1601737775"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -715,6 +1517,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
@@ -1218,19 +2060,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>317500</xdr:colOff>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>165100</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1238,7 +2583,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9EAAD089-173E-A970-CE78-01554839316C}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B175223B-803A-E581-D645-18EBD3F75B30}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1256,72 +2601,112 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>330200</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>165100</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{08FC958A-4867-42BF-B198-281AC7805E3F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="angel osorio" refreshedDate="46125.531184027779" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="8" xr:uid="{4B3AE84A-F36C-4DFE-A007-EF8622D24670}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="angel osorio" refreshedDate="46125.549112962966" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="10" xr:uid="{D1DFF387-2F43-43DE-A850-FA11D246AB50}">
   <cacheSource type="worksheet">
-    <worksheetSource name="OfficeForms.Table"/>
+    <worksheetSource ref="A1:S11" sheet="Survey"/>
   </cacheSource>
   <cacheFields count="19">
     <cacheField name="Id" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="8"/>
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="8"/>
     </cacheField>
-    <cacheField name="Start time" numFmtId="165">
-      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-04-10T12:59:11" maxDate="2026-04-12T18:01:23"/>
+    <cacheField name="Start time" numFmtId="164">
+      <sharedItems containsNonDate="0" containsDate="1" containsString="0" containsBlank="1" minDate="2026-04-10T12:59:11" maxDate="2026-04-12T18:01:23"/>
     </cacheField>
-    <cacheField name="Completion time" numFmtId="165">
-      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-04-10T13:00:31" maxDate="2026-04-12T18:02:33"/>
+    <cacheField name="Completion time" numFmtId="0">
+      <sharedItems containsNonDate="0" containsDate="1" containsString="0" containsBlank="1" minDate="2026-04-10T13:00:31" maxDate="2026-04-12T18:02:33"/>
     </cacheField>
-    <cacheField name="Time To Complete" numFmtId="45">
-      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="1899-12-30T00:00:25" maxDate="1899-12-30T00:02:29"/>
+    <cacheField name="Time To Complete" numFmtId="0">
+      <sharedItems containsNonDate="0" containsDate="1" containsString="0" containsBlank="1" minDate="1899-12-30T00:00:25" maxDate="1899-12-30T00:02:29"/>
     </cacheField>
     <cacheField name="Email" numFmtId="0">
-      <sharedItems/>
+      <sharedItems containsBlank="1"/>
     </cacheField>
     <cacheField name="Name" numFmtId="0">
-      <sharedItems/>
+      <sharedItems containsBlank="1"/>
     </cacheField>
     <cacheField name="Language" numFmtId="0">
-      <sharedItems/>
+      <sharedItems containsBlank="1"/>
     </cacheField>
     <cacheField name="How often do you visit us?" numFmtId="0">
-      <sharedItems/>
+      <sharedItems containsBlank="1"/>
     </cacheField>
     <cacheField name="What is your age group?" numFmtId="0">
-      <sharedItems/>
+      <sharedItems containsBlank="1"/>
     </cacheField>
     <cacheField name="Overall, how satisfied are you with the idea of monitoring the situation?" numFmtId="0">
-      <sharedItems/>
+      <sharedItems containsBlank="1" containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="5" maxValue="5"/>
     </cacheField>
     <cacheField name="How strongly do you agree or disagree with the following statements around this specific bar?.I am familiar with Polymarket" numFmtId="0">
-      <sharedItems/>
+      <sharedItems containsBlank="1"/>
     </cacheField>
     <cacheField name="How strongly do you agree or disagree with the following statements around this specific bar?.I am am familiar with X and it's live feed" numFmtId="0">
-      <sharedItems/>
+      <sharedItems containsBlank="1"/>
     </cacheField>
     <cacheField name="How strongly do you agree or disagree with the following statements around this specific bar?.I am familiar with a Bloomberg Terminal" numFmtId="0">
       <sharedItems containsBlank="1"/>
     </cacheField>
     <cacheField name="How strongly do you agree or disagree with the following statements around this specific bar?.I enjoy and watch sports" numFmtId="0">
-      <sharedItems/>
+      <sharedItems containsBlank="1"/>
     </cacheField>
     <cacheField name="Are you a gambler?" numFmtId="0">
-      <sharedItems count="3">
+      <sharedItems containsBlank="1" containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="3" maxValue="3" count="5">
         <s v="No"/>
         <s v="Maybe"/>
         <s v="Yes"/>
+        <n v="3"/>
+        <m/>
       </sharedItems>
     </cacheField>
     <cacheField name="How likely are you to join our rewards program?" numFmtId="0">
-      <sharedItems/>
+      <sharedItems containsBlank="1"/>
     </cacheField>
     <cacheField name="Which rewards interest you the most?" numFmtId="0">
-      <sharedItems/>
+      <sharedItems containsBlank="1"/>
     </cacheField>
     <cacheField name="How likely are you to recommend &quot;The Situation Room&quot; to a friend or colleague?" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="3" maxValue="10"/>
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="3" maxValue="10"/>
     </cacheField>
     <cacheField name="What would you add to make this a better experience?" numFmtId="0">
       <sharedItems containsBlank="1"/>
@@ -1336,7 +2721,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="8">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="10">
   <r>
     <n v="1"/>
     <d v="2026-04-10T12:59:11"/>
@@ -1505,19 +2890,61 @@
     <n v="7"/>
     <m/>
   </r>
+  <r>
+    <m/>
+    <m/>
+    <m/>
+    <d v="1899-12-30T00:01:08"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <x v="3"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="5"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <x v="4"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BBCF2208-70F1-4EA0-B6EC-D97C5D5D19CD}" name="PivotTable1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
-  <location ref="A1:A5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3DAF03DB-015F-4216-A2D9-7D05E5E3E625}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12">
+  <location ref="A1:B5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="19">
     <pivotField showAll="0"/>
-    <pivotField numFmtId="165" showAll="0"/>
-    <pivotField numFmtId="165" showAll="0"/>
-    <pivotField numFmtId="45" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -1527,10 +2954,12 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
-      <items count="4">
+      <items count="6">
+        <item h="1" x="3"/>
         <item x="1"/>
         <item x="0"/>
         <item x="2"/>
+        <item h="1" x="4"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -1544,13 +2973,13 @@
   </rowFields>
   <rowItems count="4">
     <i>
-      <x/>
-    </i>
-    <i>
       <x v="1"/>
     </i>
     <i>
       <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
     </i>
     <i t="grand">
       <x/>
@@ -1559,6 +2988,191 @@
   <colItems count="1">
     <i/>
   </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Name" fld="5" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="16">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="2">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="14" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="3">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="14" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="4">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="14" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="7" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="7" format="6">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="14" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="7" format="7">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="14" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="7" format="8">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="14" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="8" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="8" format="6">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="14" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="8" format="7">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="14" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="8" format="8">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="14" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="14" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="2">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="14" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="3">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="14" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -1575,130 +3189,129 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:S10" totalsRowCount="1">
   <autoFilter ref="A1:S9" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="19">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id" dataDxfId="19" totalsRowDxfId="15">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id" dataDxfId="32">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="id"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Start time" dataDxfId="18" totalsRowDxfId="14">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Start time" dataDxfId="31" totalsRowDxfId="13">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="startDate"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Completion time" dataDxfId="17" totalsRowDxfId="13">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Completion time" dataDxfId="30" totalsRowDxfId="12">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="submitDate"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{B540A476-BBEC-494C-A877-38FAE8082675}" name="Time To Complete" totalsRowFunction="custom" dataDxfId="16" totalsRowDxfId="12">
+    <tableColumn id="19" xr3:uid="{B540A476-BBEC-494C-A877-38FAE8082675}" name="Time To Complete" dataDxfId="29" totalsRowDxfId="11">
       <calculatedColumnFormula>C2-B2</calculatedColumnFormula>
-      <totalsRowFormula>AVERAGE(D2:D9)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="34" totalsRowDxfId="11">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="28" totalsRowDxfId="10">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="responder"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Name" dataDxfId="33" totalsRowDxfId="10">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Name" dataDxfId="27" totalsRowDxfId="9">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="responderName"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Language" dataDxfId="32" totalsRowDxfId="9">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Language" dataDxfId="26" totalsRowDxfId="8">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="submitLanguage"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="How often do you visit us?" dataDxfId="31" totalsRowDxfId="8">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="How often do you visit us?" dataDxfId="25" totalsRowDxfId="7">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rc431db57ed334582bc5c6c38fdc83c64"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="What is your age group?" dataDxfId="30" totalsRowDxfId="7">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="What is your age group?" dataDxfId="24">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r4f5121bf23274e80a9bc095f118ea8f3"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Overall, how satisfied are you with the idea of monitoring the situation?" dataDxfId="29">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Overall, how satisfied are you with the idea of monitoring the situation?" dataDxfId="23" totalsRowDxfId="6">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r86a2f8dd9f4649a0a3327d7e459e5615"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="How strongly do you agree or disagree with the following statements around this specific bar?.I am familiar with Polymarket" dataDxfId="28">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="How strongly do you agree or disagree with the following statements around this specific bar?.I am familiar with Polymarket" dataDxfId="22">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rb13b52bb0cc2432ba047e6c5eaacc8a8"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="How strongly do you agree or disagree with the following statements around this specific bar?.I am am familiar with X and it's live feed" dataDxfId="27">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="How strongly do you agree or disagree with the following statements around this specific bar?.I am am familiar with X and it's live feed" dataDxfId="21" totalsRowDxfId="5">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r19455705c32a492d9a99d0050d00afb0"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="How strongly do you agree or disagree with the following statements around this specific bar?.I am familiar with a Bloomberg Terminal" dataDxfId="26" totalsRowDxfId="6">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="How strongly do you agree or disagree with the following statements around this specific bar?.I am familiar with a Bloomberg Terminal" dataDxfId="20" totalsRowDxfId="4">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r4e39ec8855f14f32aadf2d2a6baf06c9"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="How strongly do you agree or disagree with the following statements around this specific bar?.I enjoy and watch sports" dataDxfId="25" totalsRowDxfId="5">
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="How strongly do you agree or disagree with the following statements around this specific bar?.I enjoy and watch sports" dataDxfId="19" totalsRowDxfId="3">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r0139bd1c01664392801aa6e4fb936cee"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Are you a gambler?" totalsRowLabel="=countif([Are you a gambler?], &quot;Yes&quot; )" dataDxfId="24" totalsRowDxfId="0">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Are you a gambler?" dataDxfId="18">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r018890c6500d4bfc98cfcdfd6e56b921"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="How likely are you to join our rewards program?" dataDxfId="23" totalsRowDxfId="4">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="How likely are you to join our rewards program?" dataDxfId="17" totalsRowDxfId="2">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r61d7528de8c84e17a3f681229104703d"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Which rewards interest you the most?" dataDxfId="22" totalsRowDxfId="3">
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Which rewards interest you the most?" dataDxfId="16" totalsRowDxfId="1">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r42bc9312e159432ba4335adcea04e2a6"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="How likely are you to recommend &quot;The Situation Room&quot; to a friend or colleague?" dataDxfId="21" totalsRowDxfId="2">
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="How likely are you to recommend &quot;The Situation Room&quot; to a friend or colleague?" dataDxfId="15">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rfa50d4516a6a4a769534ea482512dd0b"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="What would you add to make this a better experience?" dataDxfId="20" totalsRowDxfId="1">
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="What would you add to make this a better experience?" dataDxfId="14" totalsRowDxfId="0">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rf55a8d29143b4155ab580535c77d2f9d"/>
@@ -2030,36 +3643,52 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D8755A1-8622-4CF1-82AC-152D18EF86AD}">
-  <dimension ref="A1:A5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84273F36-284B-4888-A4D5-2BA4C7A4985C}">
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A3" s="6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" s="6" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
-        <v>65</v>
+      <c r="B5">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -2539,7 +4168,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2596,34 +4225,23 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="3"/>
+    <row r="10" spans="1:19" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="1"/>
-      <c r="D10" s="2">
-        <f>AVERAGE(D2:D9)</f>
-        <v>7.8993055376486154E-4</v>
-      </c>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="2"/>
-      <c r="M10" s="4"/>
-      <c r="N10" s="4"/>
-      <c r="O10" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="P10" s="4"/>
-      <c r="Q10" s="4"/>
-      <c r="R10" s="3"/>
-      <c r="S10" s="4"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="J10" s="7"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+      <c r="P10" s="3"/>
+      <c r="Q10" s="3"/>
+      <c r="S10" s="3"/>
     </row>
     <row r="11" spans="1:19" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="J11" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="K11" s="7"/>
-      <c r="L11" s="7"/>
+      <c r="K11" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>